<commit_message>
Major CONTRASTS update, and switch from github to gitlab.
</commit_message>
<xml_diff>
--- a/inst/extdata/LC_columns.xlsx
+++ b/inst/extdata/LC_columns.xlsx
@@ -1,25 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\aRmel_package\proteoCraft\inst\extdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anicolas\Documents\R\proteoCraft\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90FEEB55-FEF7-4873-8758-0436E38FDCE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14100"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="122">
   <si>
     <t>Name</t>
   </si>
@@ -379,14 +394,20 @@
   </si>
   <si>
     <t>Inertsil ODS4 trap column</t>
+  </si>
+  <si>
+    <t>PepSep ADVANCED</t>
+  </si>
+  <si>
+    <t>PepSep ADVANCED column (1.5 µm C18-coated particles, 25 cm * 75 µm ID, Bruker P/N 1919826)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -431,7 +452,7 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -747,8 +768,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L36"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L37"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="61.28515625" bestFit="1" customWidth="1"/>
@@ -997,7 +1018,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>120</v>
       </c>
       <c r="B8" t="s">
         <v>42</v>
@@ -1005,11 +1026,11 @@
       <c r="C8" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>45</v>
+      <c r="D8" s="4">
+        <v>25</v>
+      </c>
+      <c r="E8" s="4">
+        <v>75</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>46</v>
@@ -1022,18 +1043,16 @@
         <v>15</v>
       </c>
       <c r="J8" t="s">
-        <v>47</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>48</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="K8" s="2"/>
       <c r="L8" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="B9" t="s">
         <v>42</v>
@@ -1042,7 +1061,7 @@
         <v>43</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>45</v>
@@ -1058,10 +1077,10 @@
         <v>15</v>
       </c>
       <c r="J9" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="L9" t="s">
         <v>18</v>
@@ -1069,7 +1088,7 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B10" t="s">
         <v>42</v>
@@ -1081,7 +1100,7 @@
         <v>50</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>46</v>
@@ -1094,10 +1113,10 @@
         <v>15</v>
       </c>
       <c r="J10" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L10" t="s">
         <v>18</v>
@@ -1105,22 +1124,22 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>42</v>
       </c>
       <c r="C11" t="s">
-        <v>76</v>
-      </c>
-      <c r="D11" s="4">
-        <v>25</v>
-      </c>
-      <c r="E11" s="4">
-        <v>75</v>
+        <v>43</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>12</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="G11" s="7"/>
       <c r="H11" t="s">
@@ -1130,10 +1149,10 @@
         <v>15</v>
       </c>
       <c r="J11" t="s">
-        <v>74</v>
-      </c>
-      <c r="K11" t="s">
-        <v>68</v>
+        <v>54</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>55</v>
       </c>
       <c r="L11" t="s">
         <v>18</v>
@@ -1141,7 +1160,7 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="B12" t="s">
         <v>69</v>
@@ -1150,7 +1169,7 @@
         <v>76</v>
       </c>
       <c r="D12" s="4">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="E12" s="4">
         <v>75</v>
@@ -1166,10 +1185,10 @@
         <v>15</v>
       </c>
       <c r="J12" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="K12" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="L12" t="s">
         <v>18</v>
@@ -1177,7 +1196,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B13" t="s">
         <v>69</v>
@@ -1186,7 +1205,7 @@
         <v>76</v>
       </c>
       <c r="D13" s="4">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="E13" s="4">
         <v>75</v>
@@ -1202,10 +1221,10 @@
         <v>15</v>
       </c>
       <c r="J13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="L13" t="s">
         <v>18</v>
@@ -1213,7 +1232,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B14" t="s">
         <v>69</v>
@@ -1222,7 +1241,7 @@
         <v>76</v>
       </c>
       <c r="D14" s="4">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="E14" s="4">
         <v>75</v>
@@ -1238,10 +1257,10 @@
         <v>15</v>
       </c>
       <c r="J14" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="K14" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="L14" t="s">
         <v>18</v>
@@ -1249,37 +1268,35 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="B15" t="s">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="C15" t="s">
+        <v>76</v>
+      </c>
+      <c r="D15" s="4">
         <v>60</v>
       </c>
-      <c r="D15" s="4">
-        <v>10</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="F15" s="7">
-        <v>2.7</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>107</v>
-      </c>
+      <c r="E15" s="4">
+        <v>75</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G15" s="7"/>
       <c r="H15" t="s">
-        <v>84</v>
+        <v>14</v>
       </c>
       <c r="I15" t="s">
         <v>15</v>
       </c>
       <c r="J15" t="s">
-        <v>100</v>
-      </c>
-      <c r="K15" s="5">
-        <v>186008945</v>
+        <v>82</v>
+      </c>
+      <c r="K15" t="s">
+        <v>79</v>
       </c>
       <c r="L15" t="s">
         <v>18</v>
@@ -1287,37 +1304,37 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B16" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C16" t="s">
         <v>60</v>
       </c>
       <c r="D16" s="4">
-        <v>5</v>
-      </c>
-      <c r="E16">
-        <v>2100</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>62</v>
+        <v>10</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="F16" s="7">
+        <v>2.7</v>
       </c>
       <c r="G16" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H16" t="s">
-        <v>14</v>
+        <v>84</v>
       </c>
       <c r="I16" t="s">
         <v>15</v>
       </c>
-      <c r="J16" s="8" t="s">
-        <v>101</v>
+      <c r="J16" t="s">
+        <v>100</v>
       </c>
       <c r="K16" s="5">
-        <v>186009452</v>
+        <v>186008945</v>
       </c>
       <c r="L16" t="s">
         <v>18</v>
@@ -1325,10 +1342,10 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C17" t="s">
         <v>60</v>
@@ -1339,23 +1356,23 @@
       <c r="E17">
         <v>2100</v>
       </c>
-      <c r="F17" s="7">
-        <v>2.5</v>
+      <c r="F17" s="7" t="s">
+        <v>62</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H17" t="s">
-        <v>85</v>
+        <v>14</v>
       </c>
       <c r="I17" t="s">
         <v>15</v>
       </c>
-      <c r="J17" t="s">
-        <v>102</v>
+      <c r="J17" s="8" t="s">
+        <v>101</v>
       </c>
       <c r="K17" s="5">
-        <v>186010329</v>
+        <v>186009452</v>
       </c>
       <c r="L17" t="s">
         <v>18</v>
@@ -1363,37 +1380,37 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B18" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C18" t="s">
         <v>60</v>
       </c>
       <c r="D18" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E18">
         <v>2100</v>
       </c>
-      <c r="F18" s="7" t="s">
-        <v>62</v>
+      <c r="F18" s="7">
+        <v>2.5</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>107</v>
       </c>
       <c r="H18" t="s">
-        <v>14</v>
+        <v>85</v>
       </c>
       <c r="I18" t="s">
         <v>15</v>
       </c>
       <c r="J18" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K18" s="5">
-        <v>186009464</v>
+        <v>186010329</v>
       </c>
       <c r="L18" t="s">
         <v>18</v>
@@ -1401,22 +1418,22 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C19" t="s">
         <v>60</v>
       </c>
       <c r="D19" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E19">
-        <v>4600</v>
-      </c>
-      <c r="F19" s="7">
-        <v>2.5</v>
+        <v>2100</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>62</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>107</v>
@@ -1428,10 +1445,10 @@
         <v>15</v>
       </c>
       <c r="J19" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="K19" s="5">
-        <v>186010029</v>
+        <v>186009464</v>
       </c>
       <c r="L19" t="s">
         <v>18</v>
@@ -1439,35 +1456,37 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B20" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C20" t="s">
         <v>60</v>
       </c>
       <c r="D20" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E20">
-        <v>2100</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="G20" s="7"/>
+        <v>4600</v>
+      </c>
+      <c r="F20" s="7">
+        <v>2.5</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>107</v>
+      </c>
       <c r="H20" t="s">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="I20" t="s">
         <v>15</v>
       </c>
       <c r="J20" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K20" s="5">
-        <v>186009982</v>
+        <v>186010029</v>
       </c>
       <c r="L20" t="s">
         <v>18</v>
@@ -1475,10 +1494,10 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B21" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C21" t="s">
         <v>60</v>
@@ -1494,16 +1513,16 @@
       </c>
       <c r="G21" s="7"/>
       <c r="H21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I21" t="s">
         <v>15</v>
       </c>
       <c r="J21" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K21" s="5">
-        <v>186002878</v>
+        <v>186009982</v>
       </c>
       <c r="L21" t="s">
         <v>18</v>
@@ -1511,53 +1530,55 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="B22" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="C22" t="s">
-        <v>43</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E22" s="4"/>
-      <c r="F22" s="7"/>
+        <v>60</v>
+      </c>
+      <c r="D22" s="4">
+        <v>10</v>
+      </c>
+      <c r="E22">
+        <v>2100</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>62</v>
+      </c>
       <c r="G22" s="7"/>
       <c r="H22" t="s">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="I22" t="s">
         <v>15</v>
       </c>
       <c r="J22" t="s">
-        <v>114</v>
-      </c>
-      <c r="K22" s="2"/>
+        <v>106</v>
+      </c>
+      <c r="K22" s="5">
+        <v>186002878</v>
+      </c>
       <c r="L22" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
       <c r="B23" t="s">
-        <v>30</v>
+        <v>119</v>
       </c>
       <c r="C23" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>33</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="E23" s="4"/>
+      <c r="F23" s="7"/>
       <c r="G23" s="7"/>
       <c r="H23" t="s">
         <v>14</v>
@@ -1566,40 +1587,44 @@
         <v>15</v>
       </c>
       <c r="J23" t="s">
-        <v>34</v>
-      </c>
-      <c r="K23" s="2" t="s">
-        <v>35</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="K23" s="2"/>
       <c r="L23" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B24" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C24" t="s">
-        <v>21</v>
-      </c>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="7"/>
+        <v>10</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>33</v>
+      </c>
       <c r="G24" s="7"/>
       <c r="H24" t="s">
         <v>14</v>
       </c>
       <c r="I24" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="J24" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="K24" s="2" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="L24" t="s">
         <v>36</v>
@@ -1607,37 +1632,29 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>95</v>
+        <v>37</v>
       </c>
       <c r="B25" t="s">
-        <v>95</v>
+        <v>38</v>
       </c>
       <c r="C25" t="s">
-        <v>60</v>
-      </c>
-      <c r="D25" s="4">
-        <v>3</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="G25" s="7" t="s">
-        <v>107</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
       <c r="H25" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="I25" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="J25" t="s">
-        <v>99</v>
-      </c>
-      <c r="K25" s="5">
-        <v>186006504</v>
+        <v>39</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="L25" t="s">
         <v>36</v>
@@ -1645,43 +1662,45 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="B26" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="C26" t="s">
         <v>60</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>61</v>
+      <c r="D26" s="4">
+        <v>3</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>96</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G26" s="7"/>
+      <c r="G26" s="7" t="s">
+        <v>107</v>
+      </c>
       <c r="H26" t="s">
-        <v>14</v>
+        <v>83</v>
       </c>
       <c r="I26" t="s">
         <v>15</v>
       </c>
       <c r="J26" t="s">
-        <v>97</v>
-      </c>
-      <c r="K26" s="2" t="s">
-        <v>63</v>
+        <v>99</v>
+      </c>
+      <c r="K26" s="5">
+        <v>186006504</v>
       </c>
       <c r="L26" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B27" t="s">
         <v>72</v>
@@ -1690,7 +1709,7 @@
         <v>60</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>61</v>
@@ -1706,21 +1725,53 @@
         <v>15</v>
       </c>
       <c r="J27" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="L27" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="C28" s="6"/>
+      <c r="A28" t="s">
+        <v>71</v>
+      </c>
+      <c r="B28" t="s">
+        <v>72</v>
+      </c>
+      <c r="C28" t="s">
+        <v>60</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G28" s="7"/>
+      <c r="H28" t="s">
+        <v>14</v>
+      </c>
+      <c r="I28" t="s">
+        <v>15</v>
+      </c>
+      <c r="J28" t="s">
+        <v>98</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="L28" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C29" s="6"/>
-      <c r="J29" s="6"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C30" s="6"/>
@@ -1743,10 +1794,14 @@
       <c r="J34" s="6"/>
     </row>
     <row r="35" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C35" s="6"/>
       <c r="J35" s="6"/>
     </row>
     <row r="36" spans="3:10" x14ac:dyDescent="0.25">
       <c r="J36" s="6"/>
+    </row>
+    <row r="37" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="J37" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Large update with sweeping updates to the histones, no reps and reps with peptides only scripts. Multiple small optimisations and fixes.
</commit_message>
<xml_diff>
--- a/inst/extdata/LC_columns.xlsx
+++ b/inst/extdata/LC_columns.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anicolas\Documents\R\proteoCraft\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\aRmel_package\proteoCraft\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90FEEB55-FEF7-4873-8758-0436E38FDCE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A17AFAD-AADA-460D-BA28-E8DDD0CDFFF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="124">
   <si>
     <t>Name</t>
   </si>
@@ -400,6 +400,12 @@
   </si>
   <si>
     <t>PepSep ADVANCED column (1.5 µm C18-coated particles, 25 cm * 75 µm ID, Bruker P/N 1919826)</t>
+  </si>
+  <si>
+    <t>proteoTrap</t>
+  </si>
+  <si>
+    <t>proteoTrap (3 µm C18 particles, 50 mm * 250 µm ID, Bruker P/N 1920747)</t>
   </si>
 </sst>
 </file>
@@ -769,7 +775,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="61.28515625" bestFit="1" customWidth="1"/>
@@ -1565,20 +1571,21 @@
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>75</v>
-      </c>
       <c r="B23" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C23" t="s">
         <v>43</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="D23" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E23">
+        <v>250</v>
+      </c>
+      <c r="F23" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="E23" s="4"/>
-      <c r="F23" s="7"/>
       <c r="G23" s="7"/>
       <c r="H23" t="s">
         <v>14</v>
@@ -1587,32 +1594,30 @@
         <v>15</v>
       </c>
       <c r="J23" t="s">
-        <v>114</v>
-      </c>
-      <c r="K23" s="2"/>
+        <v>123</v>
+      </c>
+      <c r="K23" s="5">
+        <v>1920747</v>
+      </c>
       <c r="L23" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>29</v>
+        <v>75</v>
       </c>
       <c r="B24" t="s">
-        <v>30</v>
+        <v>119</v>
       </c>
       <c r="C24" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>33</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="E24" s="4"/>
+      <c r="F24" s="7"/>
       <c r="G24" s="7"/>
       <c r="H24" t="s">
         <v>14</v>
@@ -1621,40 +1626,44 @@
         <v>15</v>
       </c>
       <c r="J24" t="s">
-        <v>34</v>
-      </c>
-      <c r="K24" s="2" t="s">
-        <v>35</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="K24" s="2"/>
       <c r="L24" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C25" t="s">
-        <v>21</v>
-      </c>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="7"/>
+        <v>10</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>33</v>
+      </c>
       <c r="G25" s="7"/>
       <c r="H25" t="s">
         <v>14</v>
       </c>
       <c r="I25" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="J25" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="K25" s="2" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="L25" t="s">
         <v>36</v>
@@ -1662,37 +1671,29 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>95</v>
+        <v>37</v>
       </c>
       <c r="B26" t="s">
-        <v>95</v>
+        <v>38</v>
       </c>
       <c r="C26" t="s">
-        <v>60</v>
-      </c>
-      <c r="D26" s="4">
-        <v>3</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="F26" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="G26" s="7" t="s">
-        <v>107</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
       <c r="H26" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="I26" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="J26" t="s">
-        <v>99</v>
-      </c>
-      <c r="K26" s="5">
-        <v>186006504</v>
+        <v>39</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="L26" t="s">
         <v>36</v>
@@ -1700,43 +1701,45 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="B27" t="s">
-        <v>72</v>
+        <v>95</v>
       </c>
       <c r="C27" t="s">
         <v>60</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>61</v>
+      <c r="D27" s="4">
+        <v>3</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>96</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G27" s="7"/>
+      <c r="G27" s="7" t="s">
+        <v>107</v>
+      </c>
       <c r="H27" t="s">
-        <v>14</v>
+        <v>83</v>
       </c>
       <c r="I27" t="s">
         <v>15</v>
       </c>
       <c r="J27" t="s">
-        <v>97</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>63</v>
+        <v>99</v>
+      </c>
+      <c r="K27" s="5">
+        <v>186006504</v>
       </c>
       <c r="L27" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B28" t="s">
         <v>72</v>
@@ -1745,7 +1748,7 @@
         <v>60</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>61</v>
@@ -1761,21 +1764,53 @@
         <v>15</v>
       </c>
       <c r="J28" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="L28" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="C29" s="6"/>
+      <c r="A29" t="s">
+        <v>71</v>
+      </c>
+      <c r="B29" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" t="s">
+        <v>60</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="G29" s="7"/>
+      <c r="H29" t="s">
+        <v>14</v>
+      </c>
+      <c r="I29" t="s">
+        <v>15</v>
+      </c>
+      <c r="J29" t="s">
+        <v>98</v>
+      </c>
+      <c r="K29" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="L29" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C30" s="6"/>
-      <c r="J30" s="6"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C31" s="6"/>
@@ -1798,10 +1833,14 @@
       <c r="J35" s="6"/>
     </row>
     <row r="36" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C36" s="6"/>
       <c r="J36" s="6"/>
     </row>
     <row r="37" spans="3:10" x14ac:dyDescent="0.25">
       <c r="J37" s="6"/>
+    </row>
+    <row r="38" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="J38" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Multiple edits. Support for MSstats in protQuant.R and Stat_tests.R; pVal_check.R rewritten in depth; changed the code behind evalPlot; fixes to Volcano.plot() code.
</commit_message>
<xml_diff>
--- a/inst/extdata/LC_columns.xlsx
+++ b/inst/extdata/LC_columns.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\aRmel_package\proteoCraft\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A17AFAD-AADA-460D-BA28-E8DDD0CDFFF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{77FAA9AA-160A-41BB-A5D7-EF87C1579384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="125">
   <si>
     <t>Name</t>
   </si>
@@ -261,9 +261,6 @@
     <t>Aurora Ultimate CSI column (C18-coated particles, 25 cm * 75 C18 UHPLC column</t>
   </si>
   <si>
-    <t>experimental Inertsil ODS-4</t>
-  </si>
-  <si>
     <t>IonOptics</t>
   </si>
   <si>
@@ -378,9 +375,6 @@
     <t>15 cm monolithic capillary column (Kyoto Monotech)</t>
   </si>
   <si>
-    <t>Inertsil ODS-4 trap column (C18-coated particles, 3 cm)</t>
-  </si>
-  <si>
     <t>ID (µm)</t>
   </si>
   <si>
@@ -406,6 +400,15 @@
   </si>
   <si>
     <t>proteoTrap (3 µm C18 particles, 50 mm * 250 µm ID, Bruker P/N 1920747)</t>
+  </si>
+  <si>
+    <t>Bruker proteoTrap column</t>
+  </si>
+  <si>
+    <t>Inertsil ODS-4</t>
+  </si>
+  <si>
+    <t>Inertsil ODS-4 trap column (C18-coated particles, 3 cm, GL Sciences through Bruker)</t>
   </si>
 </sst>
 </file>
@@ -803,16 +806,16 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>118</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
@@ -832,13 +835,13 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C2" t="s">
         <v>108</v>
-      </c>
-      <c r="C2" t="s">
-        <v>109</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>57</v>
@@ -853,7 +856,7 @@
         <v>58</v>
       </c>
       <c r="J2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K2" s="2"/>
       <c r="L2" t="s">
@@ -883,7 +886,7 @@
         <v>58</v>
       </c>
       <c r="J3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" t="s">
@@ -915,7 +918,7 @@
         <v>58</v>
       </c>
       <c r="J4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" t="s">
@@ -1024,7 +1027,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B8" t="s">
         <v>42</v>
@@ -1049,7 +1052,7 @@
         <v>15</v>
       </c>
       <c r="J8" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" t="s">
@@ -1172,7 +1175,7 @@
         <v>69</v>
       </c>
       <c r="C12" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D12" s="4">
         <v>25</v>
@@ -1202,13 +1205,13 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B13" t="s">
         <v>69</v>
       </c>
       <c r="C13" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D13" s="4">
         <v>60</v>
@@ -1227,10 +1230,10 @@
         <v>15</v>
       </c>
       <c r="J13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L13" t="s">
         <v>18</v>
@@ -1238,13 +1241,13 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
         <v>69</v>
       </c>
       <c r="C14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D14" s="4">
         <v>25</v>
@@ -1263,10 +1266,10 @@
         <v>15</v>
       </c>
       <c r="J14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="K14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="L14" t="s">
         <v>18</v>
@@ -1274,13 +1277,13 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B15" t="s">
         <v>69</v>
       </c>
       <c r="C15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D15" s="4">
         <v>60</v>
@@ -1299,10 +1302,10 @@
         <v>15</v>
       </c>
       <c r="J15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="K15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="L15" t="s">
         <v>18</v>
@@ -1310,10 +1313,10 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C16" t="s">
         <v>60</v>
@@ -1328,16 +1331,16 @@
         <v>2.7</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I16" t="s">
         <v>15</v>
       </c>
       <c r="J16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="K16" s="5">
         <v>186008945</v>
@@ -1348,10 +1351,10 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B17" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C17" t="s">
         <v>60</v>
@@ -1366,7 +1369,7 @@
         <v>62</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H17" t="s">
         <v>14</v>
@@ -1375,7 +1378,7 @@
         <v>15</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K17" s="5">
         <v>186009452</v>
@@ -1386,10 +1389,10 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C18" t="s">
         <v>60</v>
@@ -1404,16 +1407,16 @@
         <v>2.5</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I18" t="s">
         <v>15</v>
       </c>
       <c r="J18" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="K18" s="5">
         <v>186010329</v>
@@ -1424,10 +1427,10 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B19" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C19" t="s">
         <v>60</v>
@@ -1442,7 +1445,7 @@
         <v>62</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H19" t="s">
         <v>14</v>
@@ -1451,7 +1454,7 @@
         <v>15</v>
       </c>
       <c r="J19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K19" s="5">
         <v>186009464</v>
@@ -1462,10 +1465,10 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C20" t="s">
         <v>60</v>
@@ -1480,7 +1483,7 @@
         <v>2.5</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H20" t="s">
         <v>14</v>
@@ -1489,7 +1492,7 @@
         <v>15</v>
       </c>
       <c r="J20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="K20" s="5">
         <v>186010029</v>
@@ -1500,10 +1503,10 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C21" t="s">
         <v>60</v>
@@ -1519,13 +1522,13 @@
       </c>
       <c r="G21" s="7"/>
       <c r="H21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I21" t="s">
         <v>15</v>
       </c>
       <c r="J21" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K21" s="5">
         <v>186009982</v>
@@ -1536,10 +1539,10 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B22" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C22" t="s">
         <v>60</v>
@@ -1555,13 +1558,13 @@
       </c>
       <c r="G22" s="7"/>
       <c r="H22" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I22" t="s">
         <v>15</v>
       </c>
       <c r="J22" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="K22" s="5">
         <v>186002878</v>
@@ -1571,8 +1574,11 @@
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>122</v>
+      </c>
       <c r="B23" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C23" t="s">
         <v>43</v>
@@ -1594,7 +1600,7 @@
         <v>15</v>
       </c>
       <c r="J23" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K23" s="5">
         <v>1920747</v>
@@ -1605,10 +1611,10 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>75</v>
+        <v>123</v>
       </c>
       <c r="B24" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C24" t="s">
         <v>43</v>
@@ -1626,7 +1632,7 @@
         <v>15</v>
       </c>
       <c r="J24" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="K24" s="2"/>
       <c r="L24" t="s">
@@ -1701,10 +1707,10 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B27" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C27" t="s">
         <v>60</v>
@@ -1713,22 +1719,22 @@
         <v>3</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>62</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I27" t="s">
         <v>15</v>
       </c>
       <c r="J27" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="K27" s="5">
         <v>186006504</v>
@@ -1764,7 +1770,7 @@
         <v>15</v>
       </c>
       <c r="J28" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="K28" s="2" t="s">
         <v>63</v>
@@ -1800,7 +1806,7 @@
         <v>15</v>
       </c>
       <c r="J29" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K29" s="2" t="s">
         <v>66</v>

</xml_diff>

<commit_message>
Updates to Volcano.plot() to make the output searchable and show individial expression data as heatmap (Z-scored) in the tooltip; Fixing some bugs for modified peptides (Excel table had no log2FC column as a result of incomplete implementation of the transition to contrasts); MSqRob implemented for modified peptides.
</commit_message>
<xml_diff>
--- a/inst/extdata/LC_columns.xlsx
+++ b/inst/extdata/LC_columns.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\aRmel_package\proteoCraft\inst\extdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="B:\home\aRmel_package\proteoCraft\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{77FAA9AA-160A-41BB-A5D7-EF87C1579384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3C4C644-76FC-4004-B877-0885D41EE7E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="130">
   <si>
     <t>Name</t>
   </si>
@@ -198,9 +198,6 @@
     <t>PepSep ULTRA</t>
   </si>
   <si>
-    <t>PepSep ULTRA column (1.5 µm C18-coated particles, 10 cm * 75 µm ID, Bruker P/N 1893484)</t>
-  </si>
-  <si>
     <t>1893484</t>
   </si>
   <si>
@@ -409,6 +406,24 @@
   </si>
   <si>
     <t>Inertsil ODS-4 trap column (C18-coated particles, 3 cm, GL Sciences through Bruker)</t>
+  </si>
+  <si>
+    <t>1919826</t>
+  </si>
+  <si>
+    <t>1.9</t>
+  </si>
+  <si>
+    <t>1893472</t>
+  </si>
+  <si>
+    <t>PepSep column (1.9 µm C18-coated particles, 10 cm * 75 µm ID, Bruker P/N 1893472)</t>
+  </si>
+  <si>
+    <t>PepSep ULTRA column (1.5 µm C18-coated particles, 25 cm * 75 µm ID, Bruker P/N 1893484)</t>
+  </si>
+  <si>
+    <t>PepSep</t>
   </si>
 </sst>
 </file>
@@ -418,7 +433,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -437,6 +452,12 @@
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -463,7 +484,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -481,6 +502,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -778,7 +806,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="61.28515625" bestFit="1" customWidth="1"/>
@@ -806,16 +834,16 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>116</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>3</v>
@@ -835,16 +863,16 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C2" t="s">
         <v>107</v>
       </c>
-      <c r="C2" t="s">
-        <v>108</v>
-      </c>
       <c r="D2" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="7"/>
@@ -853,10 +881,10 @@
         <v>14</v>
       </c>
       <c r="I2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="K2" s="2"/>
       <c r="L2" t="s">
@@ -865,16 +893,16 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C3" t="s">
         <v>43</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="7"/>
@@ -883,10 +911,10 @@
         <v>14</v>
       </c>
       <c r="I3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" t="s">
@@ -895,16 +923,16 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C4" t="s">
         <v>43</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>12</v>
@@ -915,10 +943,10 @@
         <v>14</v>
       </c>
       <c r="I4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="J4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" t="s">
@@ -1027,7 +1055,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>118</v>
+        <v>41</v>
       </c>
       <c r="B8" t="s">
         <v>42</v>
@@ -1035,11 +1063,11 @@
       <c r="C8" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="4">
-        <v>25</v>
-      </c>
-      <c r="E8" s="4">
-        <v>75</v>
+      <c r="D8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>45</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>46</v>
@@ -1052,16 +1080,18 @@
         <v>15</v>
       </c>
       <c r="J8" t="s">
-        <v>119</v>
-      </c>
-      <c r="K8" s="2"/>
+        <v>47</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>48</v>
+      </c>
       <c r="L8" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>117</v>
       </c>
       <c r="B9" t="s">
         <v>42</v>
@@ -1069,11 +1099,11 @@
       <c r="C9" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>45</v>
+      <c r="D9" s="4">
+        <v>25</v>
+      </c>
+      <c r="E9" s="4">
+        <v>75</v>
       </c>
       <c r="F9" s="7" t="s">
         <v>46</v>
@@ -1086,54 +1116,54 @@
         <v>15</v>
       </c>
       <c r="J9" t="s">
-        <v>47</v>
+        <v>118</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>48</v>
+        <v>124</v>
       </c>
       <c r="L9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>49</v>
-      </c>
-      <c r="B10" t="s">
+    <row r="10" spans="1:12" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="F10" s="7" t="s">
+      <c r="D10" s="10">
+        <v>25</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="G10" s="7"/>
-      <c r="H10" t="s">
-        <v>14</v>
-      </c>
-      <c r="I10" t="s">
-        <v>15</v>
-      </c>
-      <c r="J10" t="s">
-        <v>51</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="L10" t="s">
+      <c r="G10" s="12"/>
+      <c r="H10" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="K10" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="L10" s="9" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
         <v>42</v>
@@ -1145,7 +1175,7 @@
         <v>50</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>46</v>
@@ -1158,10 +1188,10 @@
         <v>15</v>
       </c>
       <c r="J11" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="L11" t="s">
         <v>18</v>
@@ -1169,22 +1199,22 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>129</v>
       </c>
       <c r="B12" t="s">
-        <v>69</v>
+        <v>42</v>
       </c>
       <c r="C12" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" s="4">
-        <v>25</v>
-      </c>
-      <c r="E12" s="4">
-        <v>75</v>
+        <v>43</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>12</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>62</v>
+        <v>125</v>
       </c>
       <c r="G12" s="7"/>
       <c r="H12" t="s">
@@ -1194,10 +1224,10 @@
         <v>15</v>
       </c>
       <c r="J12" t="s">
-        <v>74</v>
-      </c>
-      <c r="K12" t="s">
-        <v>68</v>
+        <v>127</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>126</v>
       </c>
       <c r="L12" t="s">
         <v>18</v>
@@ -1205,22 +1235,22 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="B13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D13" s="4">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="E13" s="4">
         <v>75</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G13" s="7"/>
       <c r="H13" t="s">
@@ -1230,10 +1260,10 @@
         <v>15</v>
       </c>
       <c r="J13" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="K13" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="L13" t="s">
         <v>18</v>
@@ -1241,22 +1271,22 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D14" s="4">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="E14" s="4">
         <v>75</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G14" s="7"/>
       <c r="H14" t="s">
@@ -1269,7 +1299,7 @@
         <v>79</v>
       </c>
       <c r="K14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="L14" t="s">
         <v>18</v>
@@ -1277,22 +1307,22 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D15" s="4">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="E15" s="4">
         <v>75</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G15" s="7"/>
       <c r="H15" t="s">
@@ -1302,10 +1332,10 @@
         <v>15</v>
       </c>
       <c r="J15" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="K15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="L15" t="s">
         <v>18</v>
@@ -1313,37 +1343,35 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="B16" t="s">
-        <v>87</v>
+        <v>68</v>
       </c>
       <c r="C16" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="4">
         <v>60</v>
       </c>
-      <c r="D16" s="4">
-        <v>10</v>
-      </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="4">
+        <v>75</v>
+      </c>
+      <c r="F16" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="F16" s="7">
-        <v>2.7</v>
-      </c>
-      <c r="G16" s="7" t="s">
-        <v>106</v>
-      </c>
+      <c r="G16" s="7"/>
       <c r="H16" t="s">
-        <v>83</v>
+        <v>14</v>
       </c>
       <c r="I16" t="s">
         <v>15</v>
       </c>
       <c r="J16" t="s">
-        <v>99</v>
-      </c>
-      <c r="K16" s="5">
-        <v>186008945</v>
+        <v>80</v>
+      </c>
+      <c r="K16" t="s">
+        <v>77</v>
       </c>
       <c r="L16" t="s">
         <v>18</v>
@@ -1351,37 +1379,37 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B17" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D17" s="4">
+        <v>10</v>
+      </c>
+      <c r="E17" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D17" s="4">
-        <v>5</v>
-      </c>
-      <c r="E17">
-        <v>2100</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>62</v>
+      <c r="F17" s="7">
+        <v>2.7</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H17" t="s">
-        <v>14</v>
+        <v>82</v>
       </c>
       <c r="I17" t="s">
         <v>15</v>
       </c>
-      <c r="J17" s="8" t="s">
-        <v>100</v>
+      <c r="J17" t="s">
+        <v>98</v>
       </c>
       <c r="K17" s="5">
-        <v>186009452</v>
+        <v>186008945</v>
       </c>
       <c r="L17" t="s">
         <v>18</v>
@@ -1389,13 +1417,13 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B18" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D18" s="4">
         <v>5</v>
@@ -1403,23 +1431,23 @@
       <c r="E18">
         <v>2100</v>
       </c>
-      <c r="F18" s="7">
-        <v>2.5</v>
+      <c r="F18" s="7" t="s">
+        <v>61</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H18" t="s">
-        <v>84</v>
+        <v>14</v>
       </c>
       <c r="I18" t="s">
         <v>15</v>
       </c>
-      <c r="J18" t="s">
-        <v>101</v>
+      <c r="J18" s="8" t="s">
+        <v>99</v>
       </c>
       <c r="K18" s="5">
-        <v>186010329</v>
+        <v>186009452</v>
       </c>
       <c r="L18" t="s">
         <v>18</v>
@@ -1427,37 +1455,37 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B19" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D19" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E19">
         <v>2100</v>
       </c>
-      <c r="F19" s="7" t="s">
-        <v>62</v>
+      <c r="F19" s="7">
+        <v>2.5</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H19" t="s">
-        <v>14</v>
+        <v>83</v>
       </c>
       <c r="I19" t="s">
         <v>15</v>
       </c>
       <c r="J19" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="K19" s="5">
-        <v>186009464</v>
+        <v>186010329</v>
       </c>
       <c r="L19" t="s">
         <v>18</v>
@@ -1465,25 +1493,25 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B20" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D20" s="4">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E20">
-        <v>4600</v>
-      </c>
-      <c r="F20" s="7">
-        <v>2.5</v>
+        <v>2100</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>61</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H20" t="s">
         <v>14</v>
@@ -1492,10 +1520,10 @@
         <v>15</v>
       </c>
       <c r="J20" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="K20" s="5">
-        <v>186010029</v>
+        <v>186009464</v>
       </c>
       <c r="L20" t="s">
         <v>18</v>
@@ -1503,35 +1531,37 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B21" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D21" s="4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E21">
-        <v>2100</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="G21" s="7"/>
+        <v>4600</v>
+      </c>
+      <c r="F21" s="7">
+        <v>2.5</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>105</v>
+      </c>
       <c r="H21" t="s">
-        <v>85</v>
+        <v>14</v>
       </c>
       <c r="I21" t="s">
         <v>15</v>
       </c>
       <c r="J21" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="K21" s="5">
-        <v>186009982</v>
+        <v>186010029</v>
       </c>
       <c r="L21" t="s">
         <v>18</v>
@@ -1539,13 +1569,13 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B22" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C22" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D22" s="4">
         <v>10</v>
@@ -1554,20 +1584,20 @@
         <v>2100</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G22" s="7"/>
       <c r="H22" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="I22" t="s">
         <v>15</v>
       </c>
       <c r="J22" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="K22" s="5">
-        <v>186002878</v>
+        <v>186009982</v>
       </c>
       <c r="L22" t="s">
         <v>18</v>
@@ -1575,55 +1605,59 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="B23" t="s">
-        <v>120</v>
+        <v>92</v>
       </c>
       <c r="C23" t="s">
-        <v>43</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>33</v>
+        <v>59</v>
+      </c>
+      <c r="D23" s="4">
+        <v>10</v>
       </c>
       <c r="E23">
-        <v>250</v>
+        <v>2100</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="G23" s="7"/>
       <c r="H23" t="s">
-        <v>14</v>
+        <v>85</v>
       </c>
       <c r="I23" t="s">
         <v>15</v>
       </c>
       <c r="J23" t="s">
-        <v>121</v>
+        <v>104</v>
       </c>
       <c r="K23" s="5">
-        <v>1920747</v>
+        <v>186002878</v>
       </c>
       <c r="L23" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B24" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C24" t="s">
         <v>43</v>
       </c>
-      <c r="D24" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="E24" s="4"/>
-      <c r="F24" s="7"/>
+      <c r="D24" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24">
+        <v>250</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>66</v>
+      </c>
       <c r="G24" s="7"/>
       <c r="H24" t="s">
         <v>14</v>
@@ -1632,32 +1666,30 @@
         <v>15</v>
       </c>
       <c r="J24" t="s">
-        <v>124</v>
-      </c>
-      <c r="K24" s="2"/>
+        <v>120</v>
+      </c>
+      <c r="K24" s="5">
+        <v>1920747</v>
+      </c>
       <c r="L24" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>29</v>
+        <v>122</v>
       </c>
       <c r="B25" t="s">
-        <v>30</v>
+        <v>116</v>
       </c>
       <c r="C25" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>33</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="E25" s="4"/>
+      <c r="F25" s="7"/>
       <c r="G25" s="7"/>
       <c r="H25" t="s">
         <v>14</v>
@@ -1666,40 +1698,44 @@
         <v>15</v>
       </c>
       <c r="J25" t="s">
-        <v>34</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>35</v>
-      </c>
+        <v>123</v>
+      </c>
+      <c r="K25" s="2"/>
       <c r="L25" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B26" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C26" t="s">
-        <v>21</v>
-      </c>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="7"/>
+        <v>10</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>33</v>
+      </c>
       <c r="G26" s="7"/>
       <c r="H26" t="s">
         <v>14</v>
       </c>
       <c r="I26" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="J26" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="L26" t="s">
         <v>36</v>
@@ -1707,37 +1743,29 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>94</v>
+        <v>37</v>
       </c>
       <c r="B27" t="s">
-        <v>94</v>
+        <v>38</v>
       </c>
       <c r="C27" t="s">
-        <v>60</v>
-      </c>
-      <c r="D27" s="4">
-        <v>3</v>
-      </c>
-      <c r="E27" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="F27" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="G27" s="7" t="s">
-        <v>106</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
       <c r="H27" t="s">
-        <v>82</v>
+        <v>14</v>
       </c>
       <c r="I27" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="J27" t="s">
-        <v>98</v>
-      </c>
-      <c r="K27" s="5">
-        <v>186006504</v>
+        <v>39</v>
+      </c>
+      <c r="K27" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="L27" t="s">
         <v>36</v>
@@ -1745,58 +1773,60 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="B28" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="C28" t="s">
-        <v>60</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E28" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D28" s="4">
+        <v>3</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="F28" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="F28" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="G28" s="7"/>
+      <c r="G28" s="7" t="s">
+        <v>105</v>
+      </c>
       <c r="H28" t="s">
-        <v>14</v>
+        <v>81</v>
       </c>
       <c r="I28" t="s">
         <v>15</v>
       </c>
       <c r="J28" t="s">
-        <v>96</v>
-      </c>
-      <c r="K28" s="2" t="s">
-        <v>63</v>
+        <v>97</v>
+      </c>
+      <c r="K28" s="5">
+        <v>186006504</v>
       </c>
       <c r="L28" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>69</v>
+      </c>
+      <c r="B29" t="s">
         <v>71</v>
       </c>
-      <c r="B29" t="s">
-        <v>72</v>
-      </c>
       <c r="C29" t="s">
+        <v>59</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E29" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="E29" s="3" t="s">
+      <c r="F29" s="7" t="s">
         <v>61</v>
-      </c>
-      <c r="F29" s="7" t="s">
-        <v>62</v>
       </c>
       <c r="G29" s="7"/>
       <c r="H29" t="s">
@@ -1806,21 +1836,53 @@
         <v>15</v>
       </c>
       <c r="J29" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="K29" s="2" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="L29" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>70</v>
+      </c>
+      <c r="B30" t="s">
+        <v>71</v>
+      </c>
+      <c r="C30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D30" s="3" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="C30" s="6"/>
+      <c r="E30" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="G30" s="7"/>
+      <c r="H30" t="s">
+        <v>14</v>
+      </c>
+      <c r="I30" t="s">
+        <v>15</v>
+      </c>
+      <c r="J30" t="s">
+        <v>96</v>
+      </c>
+      <c r="K30" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="L30" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C31" s="6"/>
-      <c r="J31" s="6"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C32" s="6"/>
@@ -1843,10 +1905,14 @@
       <c r="J36" s="6"/>
     </row>
     <row r="37" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C37" s="6"/>
       <c r="J37" s="6"/>
     </row>
     <row r="38" spans="3:10" x14ac:dyDescent="0.25">
       <c r="J38" s="6"/>
+    </row>
+    <row r="39" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="J39" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>